<commit_message>
fix: source links in text analysis + prompt/vocab refactor
- Create prompts.py as single source of truth for all LLM prompts; delete domains.py
- Fix prompt conflict: UNIVERSAL_PROMPT said NEVER use a URL as source, overriding
  the Tavily sources block; LLM now uses verbatim URLs from provided sources list
- Add load_dotenv() to auth.py and search_client.py (same root cause as JWT_SECRET bug)
- Enforce domain as Pydantic Literal; add Domain enum + kInsightTags in Flutter
- Fix domain.toUpperCase() to domain.name.toUpperCase() in core_claim_screen
- Update LLM_MODEL default to openai/gpt-oss-20b (llama-3.1-8b-instant decommissioned)
- Update developer_notes.xlsx (RBUG-013 to RBUG-017, NFR-013-015, new KDD entries)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/developer_notes.xlsx
+++ b/developer_notes.xlsx
@@ -740,7 +740,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Each evidence item includes stance (for/against/neutral) and source URL when available</t>
+          <t>Each evidence item includes stance (for/against/neutral) and source name</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Tavily web search injects real URLs into LLM prompt</t>
+          <t>Tavily web search injects real URLs; prompt enforces real org names only</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>onTapLink → launchUrl in chat_screen.dart</t>
+          <t>onTapLink â†’ launchUrl in chat_screen.dart</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1256,7 +1256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Switched to openai/gpt-oss-20b after listing live models via API</t>
+          <t>Switched model; check live models via Groq API</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Switched to openai/gpt-oss-20b</t>
+          <t>Switched to available model</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1726,6 +1726,300 @@
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>RBUG-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Backend + Frontend</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Raw Pydantic ValidationError shown to user: 'Model response didn't match expected shape: 4 validation errors...'</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>LLM returned partial JSON; Pydantic crash message passed verbatim through FastAPI 503 detail â†’ app displayed it raw</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Backend: _parse_or_retry() with setdefault defaults + retry + clean error (field names only). Frontend: _friendlyError() maps any server error to user-facing string.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>RBUG-012</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Frontend / Auth</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Analysis returned 401 Unauthorized immediately after successful login when URL arrived via share intent</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Race condition: share intent called _analyze() before AuthNotifier._restore() completed reading JWT from secure storage; token was null so Authorization header was absent</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Park URL in _pendingShareUrl; ref.listen&lt;AuthState&gt; in build() flushes it once isAuthenticated=true</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>RBUG-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Frontend / Model</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Hot reload crash: `domain.toUpperCase()` isn't defined for type Domain after Domain enum was introduced</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>domain field changed from String to Domain enum; call sites not updated</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Changed to domain.name.toUpperCase() in core_claim_screen.dart:528</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>RBUG-016</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Backend / Prompts</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Text analysis returned no source links: LLM used org names even when Tavily URLs were provided</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>UNIVERSAL_PROMPT said NEVER use a URL as a source, directly contradicting the sources block instruction to use Tavily URLs; LLM obeyed the stricter rule</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Updated UNIVERSAL_PROMPT: use verbatim URLs from provided sources list; fall back to org names/descriptors only when no sources are provided</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>RBUG-017</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Backend / Search</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>TAVILY_API_KEY not visible to search_client if imported before config.py in test/standalone contexts</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>search_client.py used os.getenv() directly without calling load_dotenv(); worked in prod via config.py import chain, but fragile</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Added load_dotenv() to search_client.py — same fix as auth.py (RBUG-014)</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>RBUG-015</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Backend / LLM</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>503 on all /analyze calls: llama-3.1-8b-instant no longer exists on Groq</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Groq decommissioned llama-3.1-8b-instant; model listed in .env but no longer available</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Checked live models via Groq API; switched LLM_MODEL to openai/gpt-oss-20b in backend/.env</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>RBUG-014</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Backend / Auth</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>RuntimeError: JWT_SECRET is not set in .env on every server start</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>auth.py reads os.getenv() directly without calling load_dotenv(); config.py loads .env but auth.py is imported independently</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Added load_dotenv() to auth.py after imports</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
@@ -1742,7 +2036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2235,6 +2529,117 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>NFR-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Data Quality</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>LLM must not hallucinate evidence source names; prompt enforces real org names or approved descriptors only</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>prompts.py UNIVERSAL_PROMPT: approved source list; NEVER invent or use URL as source</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>NFR-014</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Data Quality</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Domain category and insight tag must be from fixed vocabularies, not free-form AI text</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Domain: Pydantic Literal + Domain enum in Flutter; Tags: 10 fixed labels in prompt + kInsightTags in Dart</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>NFR-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Usability</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>LLM errors shown to user must be human-readable; never show raw Pydantic/stack traces</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>_friendlyError() in analyzing_screen.dart; _parse_or_retry() raises clean message</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2246,7 +2651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2642,12 +3047,12 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Groq</t>
+          <t>Groq (free tier)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Base URL: https://api.groq.com/openai/v1 ; Model: openai/gpt-oss-20b</t>
+          <t>Base URL: https://api.groq.com/openai/v1 ; recommended model: llama-3.1-8b-instant (low token cost)</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -2737,6 +3142,33 @@
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Dev tooling</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Git + GitHub</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Repo: github.com/YogeshNayal17/ReasoningEngine; .gitignore excludes venv, .env, *.db, MCP config</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
@@ -2753,7 +3185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2879,12 +3311,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Share intent from Android auto-fills URL and triggers analysis immediately</t>
+          <t>Share intent from Android auto-fills URL; waits for auth restore before triggering analysis (_pendingShareUrl + ref.listen&lt;AuthState&gt;)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>_applySharedUrl() + addPostFrameCallback → _analyze()</t>
+          <t>_applySharedUrl() + addPostFrameCallback â†’ _analyze()</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -2960,12 +3392,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>CoreClaimScreen: claim, credibility score, nuance score, evidence, insights, context, summary</t>
+          <t>Any LLM/server error shown as human-readable message via _friendlyError()</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>core_claim_screen.dart</t>
+          <t>analyzing_screen.dart: static _friendlyError(String raw)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -2987,12 +3419,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Evidence source URLs shown as tappable green links if they start with http</t>
+          <t>CoreClaimScreen: claim, credibility score, nuance score, evidence, insights, context, summary</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>_SourceLink widget in core_claim_screen.dart</t>
+          <t>core_claim_screen.dart</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -3009,17 +3441,17 @@
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ChatScreen: follow-up Q&amp;A with the LLM about the current analysis</t>
+          <t>Evidence source URLs shown as tappable green links if they start with http</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>chat_screen.dart, chat_controller.dart</t>
+          <t>_SourceLink widget in core_claim_screen.dart</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -3036,17 +3468,17 @@
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Assistant messages rendered as Markdown with tappable links</t>
+          <t>Domain field is typed as Domain enum (6 fixed values); falls back to Domain.general on unknown value</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>_MessageBubble uses MarkdownBody; onTapLink → launchUrl</t>
+          <t>analyze_result.dart: Domain enum + Domain.fromJson()</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -3063,17 +3495,17 @@
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Chat history loaded from file on screen init via addPostFrameCallback</t>
+          <t>Insight tag vocabulary: 10 fixed labels (High/Moderate/Low/Verified/Disputed/Unverified/Consensus/Emerging/Contested/Opinion)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>initState → chatProvider.notifier.loadFor(analysis)</t>
+          <t>analyze_result.dart: kInsightTags const set</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -3095,12 +3527,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Chat persisted after each assistant reply (unawaited)</t>
+          <t>ChatScreen: follow-up Q&amp;A with the LLM about the current analysis</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>chat_controller.dart: unawaited(chatRepository.saveFor(...))</t>
+          <t>chat_screen.dart, chat_controller.dart</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -3117,17 +3549,17 @@
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Persistence</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Saved analyses: one JSON file per user in app documents dir</t>
+          <t>Assistant messages rendered as Markdown with tappable links</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>saved_analyses_&lt;userId&gt;.json; FileSavedAnalysesRepository</t>
+          <t>_MessageBubble uses MarkdownBody; onTapLink â†’ launchUrl</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -3144,17 +3576,17 @@
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Persistence</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Chat history: one JSON file per user; keyed by claim text (120-char truncated)</t>
+          <t>Chat history loaded from file on screen init via addPostFrameCallback</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>chats_&lt;userId&gt;.json; ChatRepository</t>
+          <t>initState â†’ chatProvider.notifier.loadFor(analysis)</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -3171,17 +3603,17 @@
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Chat</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Bottom nav: Home + History always; Reasoning tab only when hasResult</t>
+          <t>Chat persisted after each assistant reply (unawaited)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>app_bottom_nav.dart: dynamic visibleTabs list</t>
+          <t>chat_controller.dart: unawaited(chatRepository.saveFor(...))</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -3198,17 +3630,17 @@
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>Persistence</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Forced light mode; ThemeMode.light in app.dart</t>
+          <t>Saved analyses: one JSON file per user in app documents dir</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>app/lib/app.dart</t>
+          <t>saved_analyses_&lt;userId&gt;.json; FileSavedAnalysesRepository</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -3225,25 +3657,106 @@
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Chat history: one JSON file per user; keyed by claim text (120-char truncated)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>chats_&lt;userId&gt;.json; ChatRepository</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Bottom nav: Home + History always; Reasoning tab only when hasResult</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>app_bottom_nav.dart: dynamic visibleTabs list</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Forced light mode; ThemeMode.light in app.dart</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>app/lib/app.dart</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>State</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>No late final fields in Notifier.build(); use ref.read() inside methods</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Prevents LateInitializationError on Riverpod rebuild</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
@@ -3260,7 +3773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3359,7 +3872,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1) Fetch URL content (if URL) → 2) Tavily search → 3) Build prompt → 4) LLM call → 5) Parse JSON response</t>
+          <t>1) Fetch URL content (if URL) â†’ 2) Tavily search â†’ 3) Build prompt â†’ 4) LLM call â†’ 5) Parse JSON response</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -3381,17 +3894,17 @@
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>LLM</t>
+          <t>Prompts</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>OpenAI Python SDK pointed at LLM_BASE_URL; works with Groq, Ollama, OpenAI</t>
+          <t>ALL LLM prompts live in prompts.py only â€” never inline in client code. build_system_prompt(domain, sources_block) composes final system prompt.</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>ollama_client.py: analyze_with_ollama()</t>
+          <t>backend/app/prompts.py</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -3408,17 +3921,17 @@
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>LLM</t>
+          <t>Prompts</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Single LLM call per analysis; domain detection merged into UNIVERSAL_PROMPT</t>
+          <t>DOMAINS tuple defines the 6 fixed categories (science/health/politics/finance/technology/general); single source of truth for backend + frontend</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>domains.py: UNIVERSAL_PROMPT</t>
+          <t>prompts.py: DOMAINS; schemas.py: Literal; analyze_result.dart: Domain enum</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -3435,17 +3948,17 @@
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>LLM</t>
+          <t>Prompts</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Groq model currently active: openai/gpt-oss-20b</t>
+          <t>Insight tag vocabulary: 10 fixed labels in UNIVERSAL_PROMPT. LLM instructed to pick from list or omit field.</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>backend/.env: LLM_MODEL</t>
+          <t>prompts.py: UNIVERSAL_PROMPT tag section</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -3462,17 +3975,17 @@
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Web search</t>
+          <t>Prompts</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Tavily API: up to 5 results fetched before LLM call; injected as sources block in system prompt</t>
+          <t>Evidence source rules: LLM must use real org/publication names (WHO, CDC, Reutersâ€¦) or approved descriptors (Scientific consensus, Medical consensusâ€¦). Never invent. Never use URL.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>search_client.py: search(), format_for_prompt()</t>
+          <t>prompts.py: UNIVERSAL_PROMPT source section</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -3489,17 +4002,17 @@
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Web search</t>
+          <t>LLM</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>LLM instructed 'do not invent URLs' in sources block</t>
+          <t>OpenAI Python SDK pointed at LLM_BASE_URL; works with Groq, Ollama, OpenAI</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>search_client.py: format_for_prompt()</t>
+          <t>ollama_client.py: analyze_with_ollama()</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -3516,17 +4029,17 @@
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Web search</t>
+          <t>LLM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Silent failure: returns [] if TAVILY_API_KEY missing or any error</t>
+          <t>Single LLM call per analysis; domain detection merged into UNIVERSAL_PROMPT</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>search_client.py</t>
+          <t>prompts.py: build_system_prompt()</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -3543,17 +4056,17 @@
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>URL fetch</t>
+          <t>LLM</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>httpx fetches og:description / og:title meta tags; falls back to &lt;title&gt;; login-gated pages use raw URL</t>
+          <t>_parse_or_retry: setdefault safe defaults â†’ try parse â†’ retry with stricter prompt â†’ raise clean error (field names only)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>reasoning.py: _fetch_url_text()</t>
+          <t>ollama_client.py: _parse_or_retry()</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -3570,17 +4083,17 @@
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Auth</t>
+          <t>Web search</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>JWT via python-jose (HS256); 30-day expiry; JWT_SECRET from .env</t>
+          <t>Tavily API: up to 5 results fetched before LLM call; injected as sources block in system prompt</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>auth.py: create_access_token()</t>
+          <t>search_client.py: search(), format_for_prompt()</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -3597,17 +4110,17 @@
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Auth</t>
+          <t>Web search</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Passwords hashed with bcrypt directly (passlib removed — bcrypt 4.x dropped __about__)</t>
+          <t>Silent failure: returns [] if TAVILY_API_KEY missing or any error; load_dotenv() called at module level</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>auth.py: hash_password(), verify_password()</t>
+          <t>search_client.py</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -3624,17 +4137,17 @@
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Database</t>
+          <t>URL fetch</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>SQLite stdlib; tables: users, daily_usage; path from VERITAS_DB_PATH env var</t>
+          <t>httpx fetches og:description / og:title meta tags; falls back to &lt;title&gt;; login-gated pages use raw URL</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>database.py: _db_path(), get_connection()</t>
+          <t>reasoning.py: _fetch_url_text()</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -3651,17 +4164,17 @@
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Daily limits</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Basic: 5 analyses / 20 questions; Nerd: 50 / 200; HTTP 429 on breach</t>
+          <t>JWT via python-jose (HS256); 30-day expiry; JWT_SECRET from .env</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Enforced in route handlers</t>
+          <t>auth.py: create_access_token()</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -3678,17 +4191,17 @@
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Mock mode</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>USE_MOCK=True skips LLM and search; returns hardcoded response</t>
+          <t>Passwords hashed with bcrypt directly (passlib removed â€” bcrypt 4.x dropped __about__)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>backend/.env</t>
+          <t>auth.py: hash_password(), verify_password()</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -3705,17 +4218,17 @@
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Error detail</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Non-200 LLM responses: 'detail' field parsed from JSON body and returned as NetworkFailure</t>
+          <t>SQLite stdlib; tables: users, daily_usage; path from VERITAS_DB_PATH env var</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>analysis_api.dart (frontend consumer)</t>
+          <t>database.py: _db_path(), get_connection()</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -3732,25 +4245,79 @@
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>Daily limits</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Basic: 5 analyses / 20 questions; Nerd: 50 / 200; HTTP 429 on breach</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>auth.py: LIMITS dict; check_and_increment_*()</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Mock mode</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>USE_MOCK=True skips LLM and search; returns hardcoded response</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>backend/.env</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>Tests</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Set VERITAS_DB_PATH + JWT_SECRET env vars before imports; _reset_db autouse fixture</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>backend/tests/test_analyze.py</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
@@ -3946,17 +4513,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>plan</t>
+          <t>is_nerd</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>TEXT DEFAULT 'basic'</t>
+          <t>INTEGER NOT NULL DEFAULT 0</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Subscription tier: basic | nerd</t>
+          <t>Subscription tier flag: 0=basic, 1=nerd</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -4011,7 +4578,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>INTEGER FOREIGN KEY → users.id</t>
+          <t>INTEGER FOREIGN KEY â†’ users.id</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -4048,7 +4615,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Usage date</t>
+          <t>Usage date; row resets next calendar day (UTC)</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -4070,7 +4637,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>analyses</t>
+          <t>analyses_count</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -4102,7 +4669,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>questions</t>
+          <t>questions_count</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -4137,7 +4704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4439,6 +5006,141 @@
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>All prompts in prompts.py only</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Single source of truth for all LLM instructions; client code should never inline prompt strings</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>build_system_prompt() composes final prompt; domains.py deleted</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Fixed domain/tag/source vocabularies enforced at all layers</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Free-form AI text in domain, insight tag, and evidence source caused inconsistent UI and hallucinated org names</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Domain: Pydantic Literal (backend) + Domain enum (Flutter). Tags: 10-label set in prompt + kInsightTags const. Sources: approved names list in UNIVERSAL_PROMPT.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>_pendingShareUrl + ref.listen&lt;AuthState&gt; for share intent race</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Share intent can arrive before AuthNotifier finishes restoring JWT from secure storage; triggering analysis with null token â†’ 401</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>URL parked in _pendingShareUrl; ref.listen flushes it once isAuthenticated=true. ref.listen in build() is the Riverpod-correct pattern for ConsumerStatefulWidget.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>_parse_or_retry: setdefault + retry + clean error</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>LLM sometimes omits required JSON fields; Pydantic ValidationError was surfacing verbatim to the user</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>setdefault fills safe defaults first; one retry with stricter prompt; on second failure raise OllamaReasoningError with field names only (not Pydantic dump)</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Groq free tier model selection</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Groq free tier: ~500k tokens/day; llama-3.1-8b-instant costs ~1,150 tokens/analysis; supports ~435 analyses/day before token cap</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Use 8b model only (not 70b); app-level limits (5/day basic) mean ~87 concurrent daily users fit within free quota with no spend</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
@@ -4591,7 +5293,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Model ID passed to LLM API</t>
+          <t>Model ID passed to LLM API; check live models at console.groq.com if 404 errors occur</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -4702,7 +5404,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>HS256 signing secret — CHANGE IN PRODUCTION</t>
+          <t>HS256 signing secret â€” CHANGE IN PRODUCTION</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -4847,17 +5549,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Groq model names change without notice; active model may become decommissioned causing 404/400 errors</t>
+          <t>Groq periodically decommissions models without notice; LLM_MODEL in .env can become stale and cause 503 errors</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Backend returns 503 / 400; check LLM_MODEL in .env</t>
+          <t>Backend returns 503; check uvicorn logs for 404 from Groq</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>List live models via Groq API and update LLM_MODEL in backend/.env</t>
+          <t>Run list_models.py script in scratchpad to find live models; update LLM_MODEL in backend/.env</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">

</xml_diff>